<commit_message>
Updates based on NanoImpact reviewer feedback
- Quick Start tab: three-step guide and worked examples, each with a
  highlighted decision-tree path and a button that opens it in the tree
- Coverage & Gaps tab: live best-tier map per matrix x monitoring step,
  matrix-specific vs. including cross-cutting documents
- Matrix filter now includes references scored in the matrix's own
  column; results flag cross-cutting (non-matrix-specific) references
- About tab: curation process, exact filter/ordering rules, when a
  lower tier fits better, how the tool grows; title/journal updated
- Glossary: document-status terms (regulation, standard, guidance, ...)
- Fix blank decision-tree diagram when it loads in a hidden tab
- Crosswalk: score SWB-MP1/MP2 (Tier 1) and De Frond 2022 (Tier 3)
  for Sub-sampling
- Smoke test: repair stale checks; verify example citations/tiers and
  Quick Start navigation end to end
</commit_message>
<xml_diff>
--- a/mnp_compass/data/crosswalk.xlsx
+++ b/mnp_compass/data/crosswalk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\methods_navigator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\mnp_compass\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED35BA5A-C0B1-4113-AA0C-36BEA9D69899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1808C267-AF69-4D68-9FB5-98F8F4FD5257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5208,7 +5208,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5483,14 +5483,47 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5512,40 +5545,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="26" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6464,75 +6463,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:54" ht="66.599999999999994" hidden="1" customHeight="1">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="109" t="s">
+      <c r="B1" s="100"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="108"/>
-      <c r="N1" s="111" t="s">
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="102"/>
+      <c r="N1" s="105" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="98"/>
+      <c r="O1" s="106"/>
       <c r="P1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Q1" s="112" t="s">
+      <c r="Q1" s="107" t="s">
         <v>40</v>
       </c>
-      <c r="R1" s="97"/>
-      <c r="S1" s="97"/>
-      <c r="T1" s="97"/>
-      <c r="U1" s="97"/>
-      <c r="V1" s="97"/>
-      <c r="W1" s="97"/>
-      <c r="X1" s="97"/>
-      <c r="Y1" s="97"/>
-      <c r="Z1" s="97"/>
-      <c r="AA1" s="97"/>
-      <c r="AB1" s="97"/>
-      <c r="AC1" s="97"/>
-      <c r="AD1" s="98"/>
-      <c r="AE1" s="113" t="s">
+      <c r="R1" s="101"/>
+      <c r="S1" s="101"/>
+      <c r="T1" s="101"/>
+      <c r="U1" s="101"/>
+      <c r="V1" s="101"/>
+      <c r="W1" s="101"/>
+      <c r="X1" s="101"/>
+      <c r="Y1" s="101"/>
+      <c r="Z1" s="101"/>
+      <c r="AA1" s="101"/>
+      <c r="AB1" s="101"/>
+      <c r="AC1" s="101"/>
+      <c r="AD1" s="106"/>
+      <c r="AE1" s="108" t="s">
         <v>41</v>
       </c>
-      <c r="AF1" s="98"/>
-      <c r="AG1" s="96" t="s">
+      <c r="AF1" s="106"/>
+      <c r="AG1" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="AH1" s="97"/>
-      <c r="AI1" s="97"/>
-      <c r="AJ1" s="98"/>
+      <c r="AH1" s="101"/>
+      <c r="AI1" s="101"/>
+      <c r="AJ1" s="106"/>
       <c r="AK1" s="15"/>
       <c r="AL1" s="16" t="s">
         <v>43</v>
       </c>
       <c r="AM1" s="78"/>
-      <c r="AN1" s="99" t="s">
+      <c r="AN1" s="110" t="s">
         <v>44</v>
       </c>
-      <c r="AO1" s="98"/>
-      <c r="AP1" s="100" t="s">
+      <c r="AO1" s="106"/>
+      <c r="AP1" s="111" t="s">
         <v>45</v>
       </c>
-      <c r="AQ1" s="98"/>
-      <c r="AR1" s="101" t="s">
+      <c r="AQ1" s="106"/>
+      <c r="AR1" s="112" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" s="102"/>
-      <c r="AT1" s="102"/>
-      <c r="AU1" s="102"/>
+      <c r="AS1" s="113"/>
+      <c r="AT1" s="113"/>
+      <c r="AU1" s="113"/>
       <c r="AV1" s="17" t="s">
         <v>44</v>
       </c>
@@ -6541,11 +6540,11 @@
       </c>
       <c r="AX1" s="19"/>
       <c r="AY1" s="19"/>
-      <c r="AZ1" s="103" t="s">
+      <c r="AZ1" s="114" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" s="104"/>
-      <c r="BB1" s="105"/>
+      <c r="BA1" s="115"/>
+      <c r="BB1" s="116"/>
     </row>
     <row r="2" spans="1:54" s="4" customFormat="1" ht="57.75" customHeight="1">
       <c r="A2" s="20" t="s">
@@ -9477,7 +9476,9 @@
       <c r="AE31" s="47">
         <v>1</v>
       </c>
-      <c r="AF31" s="47"/>
+      <c r="AF31" s="47">
+        <v>1</v>
+      </c>
       <c r="AG31" s="47">
         <v>1</v>
       </c>
@@ -11255,7 +11256,9 @@
       <c r="AC49" s="47"/>
       <c r="AD49" s="47"/>
       <c r="AE49" s="47"/>
-      <c r="AF49" s="47"/>
+      <c r="AF49" s="47">
+        <v>3</v>
+      </c>
       <c r="AG49" s="47">
         <v>3</v>
       </c>
@@ -23248,7 +23251,9 @@
       <c r="AE176" s="82">
         <v>1</v>
       </c>
-      <c r="AF176" s="82"/>
+      <c r="AF176" s="82">
+        <v>1</v>
+      </c>
       <c r="AG176" s="82">
         <v>1</v>
       </c>
@@ -24663,7 +24668,7 @@
       <c r="B191" s="3" t="s">
         <v>1458</v>
       </c>
-      <c r="C191" s="115">
+      <c r="C191" s="83">
         <v>2026</v>
       </c>
       <c r="D191" s="3" t="s">
@@ -24755,7 +24760,7 @@
       <c r="B192" s="3" t="s">
         <v>1464</v>
       </c>
-      <c r="C192" s="115">
+      <c r="C192" s="83">
         <v>2026</v>
       </c>
       <c r="D192" s="3" t="s">
@@ -24839,17 +24844,17 @@
     <row r="193" spans="1:54" ht="14.3" customHeight="1">
       <c r="A193" s="70"/>
       <c r="B193" s="3"/>
-      <c r="C193" s="115"/>
+      <c r="C193" s="83"/>
       <c r="D193" s="3"/>
       <c r="E193" s="3"/>
       <c r="F193" s="68"/>
       <c r="G193" s="90"/>
-      <c r="H193" s="114"/>
-      <c r="I193" s="116"/>
+      <c r="H193" s="96"/>
+      <c r="I193" s="97"/>
       <c r="J193" s="81"/>
       <c r="K193" s="91"/>
       <c r="L193" s="83"/>
-      <c r="M193" s="117"/>
+      <c r="M193" s="98"/>
       <c r="N193" s="82"/>
       <c r="O193" s="82"/>
       <c r="P193" s="82"/>
@@ -28191,16 +28196,16 @@
     <row r="1018" spans="1:49" ht="14.3" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AR1:AU1"/>
+    <mergeCell ref="AZ1:BB1"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="F1:M1"/>
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="Q1:AD1"/>
     <mergeCell ref="AE1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AR1:AU1"/>
-    <mergeCell ref="AZ1:BB1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E144" r:id="rId1" xr:uid="{A81C656A-0A99-4267-9649-0EEFD2B27222}"/>

</xml_diff>